<commit_message>
Clean arteri-elearning + add automation/ (E2E + unit tests from source)
</commit_message>
<xml_diff>
--- a/projects/ifl-chapter-malang/test-cases.xlsx
+++ b/projects/ifl-chapter-malang/test-cases.xlsx
@@ -513,7 +513,6 @@
           <t>Document Info</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -582,7 +581,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>76</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11">
@@ -602,9 +601,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>134</v>
-      </c>
-    </row>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -694,9 +694,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
-      </c>
-    </row>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
@@ -716,7 +717,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
@@ -726,7 +727,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
@@ -736,9 +737,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>14</v>
-      </c>
-    </row>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -852,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5113,6 +5115,1537 @@
       </c>
       <c r="K77" s="4" t="inlineStr"/>
       <c r="L77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-018</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan email mengandung SQL injection</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /masuk
+2. Isi email: ' OR 1=1--
+3. Password apa saja
+4. Klik Masuk</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>Login ditolak, error 'Format email tidak valid' (input disanitized)</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-019</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan password mengandung XSS</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>1. Isi password: &lt;script&gt;alert(1)&lt;/script&gt;
+2. Submit</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>Input di-escape, no script execution, login tetap proper</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-020</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Register dengan password terlalu pendek</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /daftar
+2. Password: 'abc'
+3. Submit</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>Validasi form gagal, error 'Password minimal 8 karakter'</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-021</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Google OAuth</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Google OAuth callback dari provider tidak dikenal</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>1. Mock callback dari domain bukan accounts.google.com</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, token google invalid</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-022</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>ProtectedRoute</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>User tanpa role akses dashboard (cookie tampering)</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>1. Modify cookie role jadi 'admin'
+2. Buka /admin/dashboards</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Backend verify role via JWT, 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-023</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Brute force: 10x login gagal bergantian</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>1. Submit password salah 10x dalam 5 menit</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Setelah 5x: 429 Too Many Requests</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>DON-017</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Donasi dengan nominal di bawah minimum</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Chatbot terbuka</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>1. Input '100' (&lt; min 10000)</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Validation feedback: 'Nominal minimum Rp 10.000'</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>DON-018</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Donasi dengan nominal di atas maksimum (1 M)</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>1. Input '10000000000' (10M, over max)</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Validation: 'Nominal maksimal Rp 10.000.000'</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>DON-019</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Midtrans</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Midtrans Snap gagal di-load (adblock)</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>1. Blokir midtrans.com di adblocker
+2. Klik Bayar</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>Loading state tampil, timeout setelah 30 detik, error message, bisa coba lagi</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>DON-020</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Midtrans</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Midtrans callback signature invalid (tampered)</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>1. Manipulasi Midtrans callback signature_key</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, callback rejected</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>DON-021</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>QRIS</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>QRIS payment expired sebelum konfirmasi</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>1. Minta QRIS
+2. Tunggu 15 menit tidak bayar</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Payment expired, kembali ke summary, bisa coba metode lain</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>DON-022</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Double Submit</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>Double click bayar (race condition)</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Di summary</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik Bayar 2x cepat</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>Hanya 1 Snap yang terbuat, idempotent (transaction_id tidak duplikat)</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>DON-023</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Donasi</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Donasi ke campaign yang sudah closed (target tercapai)</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka campaign yang sudah 100%
+2. Klik Donasi</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>Campaign marked 'Terkumpul', tombol donasi disabled atau ada warning</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>BLG-012</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>CKEditor</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>CKEditor XSS injection di konten blog</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Admin login</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>1. Add blog
+2. Konten: &lt;script&gt;alert('xss')&lt;/script&gt;
+3. Publish</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Script termakanerakan (di-sanitize) di frontend, tidak execute di browser</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>BLG-013</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>ImageKit</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>Upload file non-image (exe/pdf) sebagai cover</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik upload cover
+2. Pilih file .exe atau .pdf</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>Filter tipe file, error 'Hanya gambar yang diizinkan'</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>BLG-014</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>ImageKit</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Upload gambar &gt; 5MB</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>1. Upload gambar 10MB</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>Error: 'Ukuran file maksimal 5MB'</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>BLG-015</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Hapus blog yang sudah di-publish (tanpa draft dulu)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik Delete di blog yang sudah live</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Konfirmasi: 'Apakah Anda yakin ingin menghapus blog ini?' + warning</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>EVT-006</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>Daftar event yang sudah lewat</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka event past deadline
+2. Klik Daftar</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>Error: 'Pendaftaran sudah ditutup'</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>EVT-007</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Daftar event 2x (duplicate registration)</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>1. Daftar event
+2. Daftar lagi di event sama</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>Error: 'Anda sudah terdaftar di event ini'</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>VOL-006</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>Register volunteer tanpa nama (empty)</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>1. Isi form volunteer, kosongkan nama
+2. Submit</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>Validasi: 'Nama wajib diisi'</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>VOL-007</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>Register volunteer dengan email tidak valid</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>1. Isi email: 'bukan-email'
+2. Submit</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>Validasi: 'Format email tidak valid'</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr"/>
+      <c r="L98" s="4" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>PROF-005</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>Upload profile pic file berbahaya (.exe)</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik upload foto
+2. Pilih file .exe</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>Filter: 'Hanya file gambar yang diizinkan'</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>PROF-006</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Edit profile dengan bio &gt; 500 karakter</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>1. Edit bio 1000 karakter
+2. Save</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>Validasi: 'Bio maksimal 500 karakter'</t>
+        </is>
+      </c>
+      <c r="I100" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr"/>
+      <c r="L100" s="4" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>ADM-008</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>Akses admin endpoint langsung tanpa login</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /admin/dashboards langsung (tanpa session)</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>Redirect ke /masuk, query param ?redirect=/admin/dashboards</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>ADM-009</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Role Guard</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>User role 'bismar' akses admin-only endpoint</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>Login sebagai bismar</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /admin/dashboard/user (admin only)</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>403 Forbidden atau redirect</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr"/>
+      <c r="L102" s="4" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>ADM-010</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Role Guard</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>User role 'copywriter' akses event management</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>Login sebagai copywriter</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /admin/dashboard/event (admin+bismar only)</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>403 Forbidden atau redirect</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr"/>
+      <c r="L103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>PUB-013</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>Akses URL dengan karakter spesial (unicode, ~, $)</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /test/~$%25/xyz</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>404 halaman tampil tanpa error (tidak crash)</t>
+        </is>
+      </c>
+      <c r="I104" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="inlineStr"/>
+      <c r="L104" s="4" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>PUB-014</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>Responsive di iPad landscape (1024x768)</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka / di viewport 1024x768</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>Layout responsive, tidak ada horizontal scroll</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K105" s="4" t="inlineStr"/>
+      <c r="L105" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L77"/>

</xml_diff>

<commit_message>
Clean arteri (focus Manual+E2E+API) + add 30 API test cases IFL from be_iflchaptermalang backend
</commit_message>
<xml_diff>
--- a/projects/ifl-chapter-malang/test-cases.xlsx
+++ b/projects/ifl-chapter-malang/test-cases.xlsx
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>58</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>162</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13"/>
@@ -697,7 +697,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
@@ -740,7 +739,6 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -6659,7 +6657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9870,6 +9868,1626 @@
       <c r="K59" s="4" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
     </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-016</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>/v1/auth/refresh-token</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Refresh JWT token menggunakan refresh_token</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>User has refresh_token</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>?refresh_token=valid_refresh_token</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, new access_token + refresh_token pair</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr"/>
+      <c r="L60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-017</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>/v1/auth/email/resend</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Resend email verification</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>User registered but not verified</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>{"email": "user@test.com"}</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, verification email resent</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-018</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>/v1/auth/logout</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Logout — invalidate current token</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>(with valid token)</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, token invalidated</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr"/>
+      <c r="L62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-019</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>/v1/auth/password/email</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Send forgot password link to email</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>User registered</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>{"email": "user@test.com"}</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, reset link sent</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-020</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>/v1/auth/notice/emailNotVerified</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Get email not verified notice page</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>(no params)</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, notice page content</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>API-PROF-001</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>/v1/profile/update-password</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>Update current user password</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>{"current_password": "old123", "new_password": "new123!"}</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, password updated</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>API-PROF-002</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>/v1/profile/edit</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Update profile (name, phone, avatar via ImageKit)</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>{"name": "Updated Name", "phone": "08123456789"}</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, profile updated</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>API-COMM-001</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>/v1/blog/{blog_id}/comment</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Get list comments for a blog post</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>/v1/blog/1/comment</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, list comments</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>API-COMM-002</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>/v1/blog/{blog_id}/comment</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Add comment to a blog post</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>{"comment": "Great article!"}</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, comment added</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>API-COMM-003</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>/v1/blog/{blog_id}/comment/{comment_id}</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Reply to a comment</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Comment exists</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>{"comment": "Thanks for your feedback!"}</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, reply added</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>API-COMM-004</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>/v1/comment/{comment_id}/toggle-like</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Toggle like on a comment</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {liked: true/false, total_likes}</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>API-COMM-005</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>/v1/blog/{blog_id}/toggle-like</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>Toggle like on a blog post</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {liked: true/false, total_likes}</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>API-EVT-008</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>/v1/event</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Create event (admin only)</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Login as admin</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "...", "date": "2026-12-01", "location": "...", "description": "..."}</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, event_id</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>API-EVT-009</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>/v1/event/{id}</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Update event with file upload (admin)</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Event exists</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>multipart: _method=PUT, title="Updated", cover=@image.jpg</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, event updated</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>API-EVT-010</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>/v1/event/{id}</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Delete event (admin only)</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Event exists</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, event deleted</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>API-TRANS-001</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>/v1/transaction/create/{campaignSlug}</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Create transaction via Midtrans</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>{"amount": 50000, "payment_method": "bank_transfer", "donor_name": "Anonymous"}</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, {transaction_id, snap_token, payment_url}</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>API-TRANS-002</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>/v1/transaction/callback</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Midtrans payment callback</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Valid signature from Midtrans</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>{"transaction_id": "...", "transaction_status": "settlement", "signature_key": "..."}</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, donation status updated</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr"/>
+      <c r="L76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>API-TRANS-003</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>/v1/transaction/status/{id}</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Check transaction status</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>/v1/transaction/status/123</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {status, gross_amount, payment_type}</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>API-VOL-005</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>/v1/volunteer/referral-code/validate/{code}</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Validate referral code</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>/v1/volunteer/referral-code/validate/REF123</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {valid: true, referral: {code, discount}}</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>API-VOL-006</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>/v1/volunteer/registration/form-data</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Get volunteer registration form data (dropdowns, options)</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>(with valid token)</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {events: [...], skills: [...], ...}</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>API-VOL-007</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>/v1/volunteer/registration/my-registration</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Get my volunteer registration status</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>User already registered</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>(with valid token)</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {registration: {status, event, ...}}</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-006</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/volunteer-registrations</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>List all volunteer registrations (admin)</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Login as admin</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>?status=pending&amp;page=1</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, list with pagination</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-007</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/volunteer-registrations/{id}/status</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Approve/reject volunteer registration</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Registration exists</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>{"status": "approved"}</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, status updated</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-008</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/volunteer-registrations/bulk-update-status</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Bulk approve/reject registrations</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>{"ids": [1,2,3], "status": "approved"}</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {updated: 3}</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-009</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/volunteer-registrations/export</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Export volunteer registrations to CSV/Excel</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Login as admin</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>?status=approved</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, file download (CSV/XLSX)</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-010</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/{id}</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Get user by ID (admin)</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Login as admin</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/5</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, {id, name, email, role, ...}</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-011</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/{id}</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Update user (admin)</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>{"name": "...", "role": "bismar"}</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, user updated</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-012</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/{id}</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Delete user (admin)</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, user deleted (soft delete)</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-013</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/donations/pending</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>List pending manual donations (admin)</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>(with admin token)</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, list pending donations requiring manual approval</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>API-ADM-014</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>/v1/admin/donations/{id}/approve</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>Approve pending manual donation (admin)</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Donation is pending</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>200 OK, donation approved, status updated</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>